<commit_message>
chore: regenerate template binaries (auto)
</commit_message>
<xml_diff>
--- a/public/downloads/appliance-repair-invoice-template.xlsx
+++ b/public/downloads/appliance-repair-invoice-template.xlsx
@@ -534,7 +534,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F34"/>
+  <dimension ref="A1:G40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -543,6 +543,7 @@
     <col width="16" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="10" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -690,6 +691,11 @@
           <t>Amount ($)</t>
         </is>
       </c>
+      <c r="G16" s="7" t="inlineStr">
+        <is>
+          <t>Taxable</t>
+        </is>
+      </c>
     </row>
     <row r="17" ht="18" customHeight="1">
       <c r="A17" s="9" t="n">
@@ -715,6 +721,9 @@
         <f>C17*E17</f>
         <v/>
       </c>
+      <c r="G17" s="9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="18" ht="18" customHeight="1">
       <c r="A18" s="9" t="n">
@@ -740,6 +749,9 @@
         <f>C18*E18</f>
         <v/>
       </c>
+      <c r="G18" s="9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="19" ht="18" customHeight="1">
       <c r="A19" s="9" t="n">
@@ -765,6 +777,9 @@
         <f>C19*E19</f>
         <v/>
       </c>
+      <c r="G19" s="9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="20" ht="18" customHeight="1">
       <c r="A20" s="9" t="n">
@@ -790,6 +805,9 @@
         <f>C20*E20</f>
         <v/>
       </c>
+      <c r="G20" s="9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="21" ht="18" customHeight="1">
       <c r="A21" s="9" t="n">
@@ -815,6 +833,9 @@
         <f>C21*E21</f>
         <v/>
       </c>
+      <c r="G21" s="9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="22" ht="18" customHeight="1">
       <c r="A22" s="9" t="n">
@@ -840,6 +861,9 @@
         <f>C22*E22</f>
         <v/>
       </c>
+      <c r="G22" s="9" t="b">
+        <v>1</v>
+      </c>
     </row>
     <row r="24">
       <c r="D24" s="3" t="inlineStr">
@@ -872,7 +896,7 @@
         </is>
       </c>
       <c r="F26" s="11">
-        <f>IF(E25="","",ROUND(F24*E25,2))</f>
+        <f>IF(E25="","",ROUND(SUMPRODUCT(($G$17:$G$22=TRUE)*F17:F22)*E25,2))</f>
         <v/>
       </c>
     </row>
@@ -887,43 +911,106 @@
         <v/>
       </c>
     </row>
-    <row r="29" ht="30" customHeight="1">
-      <c r="A29" s="3" t="inlineStr">
+    <row r="28">
+      <c r="C28" s="13" t="inlineStr">
+        <is>
+          <t>enter if collected</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>DEPOSIT RECEIVED</t>
+        </is>
+      </c>
+      <c r="F28" s="11" t="n"/>
+    </row>
+    <row r="29">
+      <c r="C29" s="13" t="inlineStr">
+        <is>
+          <t>enter if any</t>
+        </is>
+      </c>
+      <c r="D29" s="3" t="inlineStr">
+        <is>
+          <t>AMOUNT PAID</t>
+        </is>
+      </c>
+      <c r="F29" s="11" t="n"/>
+    </row>
+    <row r="30">
+      <c r="D30" s="15" t="inlineStr">
+        <is>
+          <t>BALANCE DUE</t>
+        </is>
+      </c>
+      <c r="F30" s="16">
+        <f>F27-IF(ISNUMBER(F28),F28,0)-IF(ISNUMBER(F29),F29,0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="32" ht="30" customHeight="1">
+      <c r="A32" s="3" t="inlineStr">
         <is>
           <t>PAYMENT TERMS:</t>
         </is>
       </c>
-      <c r="B29" s="4" t="inlineStr">
+      <c r="B32" s="4" t="inlineStr">
         <is>
           <t>Payment due at time of service. Parts carry a 90-day warranty; labor is guaranteed for 90 days.</t>
         </is>
       </c>
     </row>
-    <row r="30">
-      <c r="A30" s="3" t="inlineStr">
+    <row r="33">
+      <c r="A33" s="3" t="inlineStr">
         <is>
           <t>NOTES:</t>
         </is>
       </c>
-      <c r="B30" s="4" t="inlineStr">
+      <c r="B33" s="4" t="inlineStr">
         <is>
           <t>Thank you for your business. Diagnostic fee is waived if you approve the repair. Brand and model should be listed on the work order for warranty tracking.</t>
         </is>
       </c>
     </row>
-    <row r="32">
-      <c r="A32" s="17" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
+        <is>
+          <t>PAYMENT:</t>
+        </is>
+      </c>
+      <c r="B34" s="4" t="inlineStr">
+        <is>
+          <t>Make checks payable to: ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="B35" s="4" t="inlineStr">
+        <is>
+          <t>Card / Venmo / Zelle: ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="B36" s="4" t="inlineStr">
+        <is>
+          <t>Pay online: ______</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="17" t="inlineStr">
         <is>
           <t>Template for informational purposes only; does not constitute legal, tax, or accounting advice. Requirements vary by state — verify with your licensing authority and CPA/attorney.</t>
         </is>
       </c>
     </row>
-    <row r="33"/>
-    <row r="34"/>
+    <row r="39"/>
+    <row r="40"/>
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="A1:F1"/>
-    <mergeCell ref="A32:F34"/>
+    <mergeCell ref="A38:F40"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>